<commit_message>
Budget re-cut to match the submitted proposal; late seed files
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/application/ama-amoedo-2026/NKM_Budget_AmaAmoedo_2026.xlsx
+++ b/application/ama-amoedo-2026/NKM_Budget_AmaAmoedo_2026.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,11 +53,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
       <sz val="10"/>
     </font>
     <font>
@@ -102,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,11 +116,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -493,12 +487,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -507,14 +501,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>New Kinds of Minds: A Global Atlas of Neurodiversity</t>
+          <t>New Kinds of Minds</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Phase I: Mapping Latin American Neurodiversity. Budget, January to December 2027, in US dollars.</t>
+          <t>A participatory digital artwork about the diversity of human experience. Budget, January to December 2027, in US dollars.</t>
         </is>
       </c>
     </row>
@@ -560,24 +554,24 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Research and mapping</t>
+          <t>Contributions</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Regional mapping contributors</t>
+          <t>Commissioned and licensed contributions</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Two contributors (Brazil; Spanish-speaking Latin America), ~6 months part-time research and verification each</t>
+          <t>Fees to Latin American artists and initiatives for sound pieces, drawings, photographs, short films, performances and writing (about 25 contributions, average US$140)</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>1300</v>
+        <v>140</v>
       </c>
       <c r="F6" s="5">
         <f>D6*E6</f>
@@ -587,24 +581,24 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Community participation</t>
+          <t>Contributions</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Advisory circle honoraria</t>
+          <t>Recorded conversations</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Six neurodivergent advisors from mapped initiatives, two taxonomy sessions plus consultation</t>
+          <t>Participant fees, transcription and subtitling for about 10 recorded conversations with willing participants</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F7" s="5">
         <f>D7*E7</f>
@@ -614,24 +608,24 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Community participation</t>
+          <t>Artistic production</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Participant-written descriptions and testimonies</t>
+          <t>Sound composition and visual environment</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Fees for initiatives writing their own entries and short testimonies (approx. 25 at US$20)</t>
+          <t>Composition and production of the navigable sonic and visual environment around the contributions</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>500</v>
+        <v>1800</v>
       </c>
       <c r="F8" s="5">
         <f>D8*E8</f>
@@ -641,24 +635,24 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Artistic development</t>
+          <t>Artistic production</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Interface and visualization development</t>
+          <t>Interface development</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Trilingual interface, network field, visual system extension</t>
+          <t>Building the exploratory paths, contribution pages and media playback alongside the geographic navigation</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="F9" s="5">
         <f>D9*E9</f>
@@ -668,24 +662,24 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Artistic development</t>
+          <t>Translation and accessibility</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Data-visual essays</t>
+          <t>Translation</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Two commissioned essays on patterns in the Latin American mapping (US$350 each)</t>
+          <t>Portuguese and Spanish navigation, translation of contributions and summaries</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>350</v>
+        <v>700</v>
       </c>
       <c r="F10" s="5">
         <f>D10*E10</f>
@@ -695,24 +689,24 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Translation and accessibility</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Accessibility review</t>
+          <t>Accessibility review and implementation</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Review by a neurodivergent-led accessibility consultancy (keyboard, screen reader, cognitive load, motion, plain language)</t>
+          <t>Review of the media layer with neurodivergent consultants; captions, transcripts, motion and sound controls</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="F11" s="5">
         <f>D11*E11</f>
@@ -722,24 +716,24 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Public presentation</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Accessibility implementation</t>
+          <t>Participant review and public presentation</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Implementing review findings across map, index, entry and contribution flows</t>
+          <t>Online review sessions with contributors and a public online presentation, with captioning</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>400</v>
+        <v>700</v>
       </c>
       <c r="F12" s="5">
         <f>D12*E12</f>
@@ -749,24 +743,24 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Translation</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Translation and localization</t>
+          <t>Hosting, media storage and domain</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Interface strings and 300+ summaries in Portuguese, Spanish and English</t>
+          <t>Twelve months of hosting, audio and video storage, backups</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="F13" s="5">
         <f>D13*E13</f>
@@ -776,24 +770,24 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Public programming</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Online gatherings</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Three gatherings among mapped initiatives: facilitation, live captioning, interpretation</t>
+          <t>Screen recordings, stills, written account of the method, outreach materials</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="F14" s="5">
         <f>D14*E14</f>
@@ -803,24 +797,24 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Public programming</t>
+          <t>Contingency</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Launch program</t>
+          <t>Transfer, currency and contingency</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Public online launch of dataset 1.0 with invited initiatives</t>
+          <t>Bank transfer fees, currency conversion, unforeseen production costs</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="F15" s="5">
         <f>D15*E15</f>
@@ -828,277 +822,152 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Domain, hosting, database and API</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Twelve months of infrastructure, geocoding and backups</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>500</v>
-      </c>
-      <c r="F16" s="5">
-        <f>D16*E16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Documentation and communication</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Short video, screenshots, printed dossier, outreach to initiatives and research groups</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>500</v>
-      </c>
-      <c r="F17" s="5">
-        <f>D17*E17</f>
+      <c r="A16" s="6" t="inlineStr"/>
+      <c r="B16" s="6" t="inlineStr"/>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr"/>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="7">
+        <f>SUM(F6:F15)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Bank transfer and currency costs</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Transfer fees and conversion on the award and on payments to collaborators</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>200</v>
-      </c>
-      <c r="F18" s="5">
-        <f>D18*E18</f>
-        <v/>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>By category</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr"/>
-      <c r="B19" s="6" t="inlineStr"/>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr"/>
-      <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="7">
-        <f>SUM(F6:F18)</f>
-        <v/>
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Contributions</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Artistic production</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="n">
+        <v>2400</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>0.24</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>By category</t>
-        </is>
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Translation and accessibility</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>0.13</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Research and mapping</t>
+          <t>Public presentation</t>
         </is>
       </c>
       <c r="E22" s="10" t="n">
-        <v>2600</v>
+        <v>700</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>0.26</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Community participation</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E23" s="10" t="n">
-        <v>1700</v>
+        <v>300</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>0.17</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Artistic development</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E24" s="10" t="n">
-        <v>1700</v>
+        <v>400</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>0.17</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Contingency</t>
         </is>
       </c>
       <c r="E25" s="10" t="n">
-        <v>1100</v>
+        <v>400</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>Translation</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="n">
-        <v>900</v>
-      </c>
-      <c r="F26" s="11" t="n">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>Public programming</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="n">
-        <v>800</v>
-      </c>
-      <c r="F27" s="11" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="E28" s="10" t="n">
-        <v>500</v>
-      </c>
-      <c r="F28" s="11" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="n">
-        <v>500</v>
-      </c>
-      <c r="F29" s="11" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="E30" s="10" t="n">
-        <v>200</v>
-      </c>
-      <c r="F30" s="11" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>People, participation and artistic production share</t>
-        </is>
-      </c>
-      <c r="F31" s="11" t="n">
-        <v>0.88</v>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="13" t="inlineStr">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="14" t="inlineStr">
-        <is>
-          <t>Infrastructure already exists (static site, open dataset, submissions service) and is not funded retroactively; the grant buys the collective year of work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="14" t="inlineStr">
-        <is>
-          <t>All collaborator payments are fees for work performed during the project period. No personal expenses, debts, legal costs or fundraising events are included.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>The award is received as a single transfer to the applicant's account; contributors and advisors are paid from it on delivery of agreed work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="14" t="inlineStr">
-        <is>
-          <t>Figures are estimates in US dollars; exchange-rate variation is absorbed by the contingency line and, if needed, by the documentation line.</t>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>The platform and its first 471 entries exist already and are not funded retroactively. The grant funds the collective artwork: paid contributions, conversations, and the environment that holds them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>All payments to contributors are fees for work created or licensed during the project period. No personal expenses, debts, legal costs or fundraising events are included.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Figures are estimates in US dollars; exchange-rate variation is absorbed by the contingency line.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A35:F35"/>
+  <mergeCells count="4">
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A27:F27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>